<commit_message>
correzione errore rrahmani a
</commit_message>
<xml_diff>
--- a/downloads/Giocatori_Titolari_Rigoristi_2026_27.xlsx
+++ b/downloads/Giocatori_Titolari_Rigoristi_2026_27.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matortor\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39E6792C-0B77-4964-A005-D490EF9DC530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86561ED5-1084-43C9-8590-557D69CF801B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1007,7 +1007,7 @@
     <t>Halhal</t>
   </si>
   <si>
-    <t>Rrahmani AI.</t>
+    <t>Rrahmani A</t>
   </si>
 </sst>
 </file>

</xml_diff>